<commit_message>
Merge 4.0.6/4.0.7 into 5.0
</commit_message>
<xml_diff>
--- a/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
+++ b/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ccs\BCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ccs\BCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9F6EC0-2F2F-4CCB-BD1C-F954EC71A52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2553FA00-BEA9-4BC5-86DD-DAE52C474F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23730" yWindow="2610" windowWidth="21825" windowHeight="13170" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -21,9 +21,6 @@
     <sheet name="BCS-electricity" sheetId="9" r:id="rId6"/>
     <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId7"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">About!$A$11</definedName>
     <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
@@ -61,6 +58,9 @@
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="113">
   <si>
     <t>Source:</t>
   </si>
@@ -82,9 +82,6 @@
     <t>None needed</t>
   </si>
   <si>
-    <t>2022 to 2012 USD</t>
-  </si>
-  <si>
     <t>This variable captures any BAU subsidies for CCS, specified in dollars per ton captured.</t>
   </si>
   <si>
@@ -331,9 +328,6 @@
     <t>values for industry only to reflect the duration multiplier.</t>
   </si>
   <si>
-    <t>Unit: dimensionless (% of project cost)</t>
-  </si>
-  <si>
     <t>hard coal</t>
   </si>
   <si>
@@ -404,6 +398,15 @@
   </si>
   <si>
     <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>2025 to 2012 USD (model OCCF, InputData/web-app/OCCF)</t>
+  </si>
+  <si>
+    <t>https://www.bls.gov/data/inflation_calculator.htm</t>
+  </si>
+  <si>
+    <t>*26 U.S.C. 45Q(b)(1): inflation adjustment applies to taxable years beginning after 2026, substituting 2025 for 1990 - so the $85 is in 2025 dollars and we use the 2025 currency year to adjust to 2012 $. Factor matches the model OCCF (0.713109). Electricity CCS receives the credit through 2035: construction must begin before 1/1/2033 (45Q(d)), plus the 3-year construction timeline below.</t>
   </si>
 </sst>
 </file>
@@ -510,34 +513,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="About"/>
-      <sheetName val="Calculations"/>
-      <sheetName val="BCS-BCS"/>
-      <sheetName val="BCS-DoSfCS"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3">
-        <row r="2">
-          <cell r="B2">
-            <v>12</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -835,12 +810,12 @@
     <col min="4" max="4" width="30.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -848,85 +823,93 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
-        <v>0.78500000000000003</v>
+        <v>0.71310899999999999</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="C9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="5">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
         <v>21</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>22</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" s="8">
         <v>229.59399999999999</v>
@@ -943,7 +926,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B21" s="8">
         <v>232.95699999999999</v>
@@ -960,7 +943,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="8">
         <v>236.73599999999999</v>
@@ -977,7 +960,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="8">
         <v>237.017</v>
@@ -994,7 +977,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="8">
         <v>240.00700000000001</v>
@@ -1011,7 +994,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="8">
         <v>245.12</v>
@@ -1028,7 +1011,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="8">
         <v>251.107</v>
@@ -1045,7 +1028,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="8">
         <v>255.65700000000001</v>
@@ -1062,7 +1045,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" s="8">
         <v>258.81099999999998</v>
@@ -1079,7 +1062,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B29" s="8">
         <v>270.97000000000003</v>
@@ -1096,7 +1079,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30" s="8">
         <v>292.65499999999997</v>
@@ -1113,7 +1096,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B31" s="8">
         <v>304.702</v>
@@ -1124,7 +1107,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B32">
         <v>313.68900000000002</v>
@@ -1139,7 +1122,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B33" s="7">
         <f>B32/(1-$B$37/100)</f>
@@ -1152,7 +1135,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" s="7">
         <f>B33/(1-$B$37/100)</f>
@@ -1165,7 +1148,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="7">
         <f>B34/(1-$B$37/100)</f>
@@ -1178,38 +1161,38 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B37">
         <v>2.5</v>
       </c>
       <c r="C37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1230,20 +1213,20 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1357,7 +1340,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="6">
         <f>About!B11</f>
@@ -1366,7 +1349,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>20</v>
@@ -1374,7 +1357,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>12</v>
@@ -1382,7 +1365,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="6">
         <f>B1*B3/B2</f>
@@ -1496,7 +1479,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1596,142 +1579,142 @@
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3">
-        <f>IFERROR(IF(A3=1,1,INDEX($B$2:$AE$2,MATCH((B1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(A3=1,1,INDEX($B$2:$AE$2,MATCH((B1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="C3">
-        <f>IFERROR(IF(B3=1,1,INDEX($B$2:$AE$2,MATCH((C1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(B3=1,1,INDEX($B$2:$AE$2,MATCH((C1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="D3">
-        <f>IFERROR(IF(C3=1,1,INDEX($B$2:$AE$2,MATCH((D1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(C3=1,1,INDEX($B$2:$AE$2,MATCH((D1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="E3">
-        <f>IFERROR(IF(D3=1,1,INDEX($B$2:$AE$2,MATCH((E1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(D3=1,1,INDEX($B$2:$AE$2,MATCH((E1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="F3">
-        <f>IFERROR(IF(E3=1,1,INDEX($B$2:$AE$2,MATCH((F1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(E3=1,1,INDEX($B$2:$AE$2,MATCH((F1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="G3">
-        <f>IFERROR(IF(F3=1,1,INDEX($B$2:$AE$2,MATCH((G1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(F3=1,1,INDEX($B$2:$AE$2,MATCH((G1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="H3">
-        <f>IFERROR(IF(G3=1,1,INDEX($B$2:$AE$2,MATCH((H1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(G3=1,1,INDEX($B$2:$AE$2,MATCH((H1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="I3">
-        <f>IFERROR(IF(H3=1,1,INDEX($B$2:$AE$2,MATCH((I1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(H3=1,1,INDEX($B$2:$AE$2,MATCH((I1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="J3">
-        <f>IFERROR(IF(I3=1,1,INDEX($B$2:$AE$2,MATCH((J1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(I3=1,1,INDEX($B$2:$AE$2,MATCH((J1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="K3">
-        <f>IFERROR(IF(J3=1,1,INDEX($B$2:$AE$2,MATCH((K1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(J3=1,1,INDEX($B$2:$AE$2,MATCH((K1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="L3">
-        <f>IFERROR(IF(K3=1,1,INDEX($B$2:$AE$2,MATCH((L1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(K3=1,1,INDEX($B$2:$AE$2,MATCH((L1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="M3">
-        <f>IFERROR(IF(L3=1,1,INDEX($B$2:$AE$2,MATCH((M1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(L3=1,1,INDEX($B$2:$AE$2,MATCH((M1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="N3">
-        <f>IFERROR(IF(M3=1,1,INDEX($B$2:$AE$2,MATCH((N1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(M3=1,1,INDEX($B$2:$AE$2,MATCH((N1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="O3">
-        <f>IFERROR(IF(N3=1,1,INDEX($B$2:$AE$2,MATCH((O1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(N3=1,1,INDEX($B$2:$AE$2,MATCH((O1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="P3">
-        <f>IFERROR(IF(O3=1,1,INDEX($B$2:$AE$2,MATCH((P1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(O3=1,1,INDEX($B$2:$AE$2,MATCH((P1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="Q3">
-        <f>IFERROR(IF(P3=1,1,INDEX($B$2:$AE$2,MATCH((Q1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(P3=1,1,INDEX($B$2:$AE$2,MATCH((Q1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="R3">
-        <f>IFERROR(IF(Q3=1,1,INDEX($B$2:$AE$2,MATCH((R1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(Q3=1,1,INDEX($B$2:$AE$2,MATCH((R1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="S3">
-        <f>IFERROR(IF(R3=1,1,INDEX($B$2:$AE$2,MATCH((S1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(R3=1,1,INDEX($B$2:$AE$2,MATCH((S1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="T3">
-        <f>IFERROR(IF(S3=1,1,INDEX($B$2:$AE$2,MATCH((T1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(S3=1,1,INDEX($B$2:$AE$2,MATCH((T1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="U3">
-        <f>IFERROR(IF(T3=1,1,INDEX($B$2:$AE$2,MATCH((U1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(T3=1,1,INDEX($B$2:$AE$2,MATCH((U1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="V3">
-        <f>IFERROR(IF(U3=1,1,INDEX($B$2:$AE$2,MATCH((V1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(U3=1,1,INDEX($B$2:$AE$2,MATCH((V1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="W3">
-        <f>IFERROR(IF(V3=1,1,INDEX($B$2:$AE$2,MATCH((W1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(V3=1,1,INDEX($B$2:$AE$2,MATCH((W1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0</v>
       </c>
       <c r="X3">
-        <f>IFERROR(IF(W3=1,1,INDEX($B$2:$AE$2,MATCH((X1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(W3=1,1,INDEX($B$2:$AE$2,MATCH((X1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0.2</v>
       </c>
       <c r="Y3">
-        <f>IFERROR(IF(X3=1,1,INDEX($B$2:$AE$2,MATCH((Y1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(X3=1,1,INDEX($B$2:$AE$2,MATCH((Y1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0.4</v>
       </c>
       <c r="Z3">
-        <f>IFERROR(IF(Y3=1,1,INDEX($B$2:$AE$2,MATCH((Z1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(Y3=1,1,INDEX($B$2:$AE$2,MATCH((Z1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0.60000000000000009</v>
       </c>
       <c r="AA3">
-        <f>IFERROR(IF(Z3=1,1,INDEX($B$2:$AE$2,MATCH((AA1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(Z3=1,1,INDEX($B$2:$AE$2,MATCH((AA1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>0.8</v>
       </c>
       <c r="AB3">
-        <f>IFERROR(IF(AA3=1,1,INDEX($B$2:$AE$2,MATCH((AB1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(AA3=1,1,INDEX($B$2:$AE$2,MATCH((AB1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>1</v>
       </c>
       <c r="AC3">
-        <f>IFERROR(IF(AB3=1,1,INDEX($B$2:$AE$2,MATCH((AC1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(AB3=1,1,INDEX($B$2:$AE$2,MATCH((AC1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>1</v>
       </c>
       <c r="AD3">
-        <f>IFERROR(IF(AC3=1,1,INDEX($B$2:$AE$2,MATCH((AD1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(AC3=1,1,INDEX($B$2:$AE$2,MATCH((AD1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>1</v>
       </c>
       <c r="AE3">
-        <f>IFERROR(IF(AD3=1,1,INDEX($B$2:$AE$2,MATCH((AE1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <f>IFERROR(IF(AD3=1,1,INDEX($B$2:$AE$2,MATCH((AE1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
@@ -1747,17 +1730,17 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B11">
         <v>14</v>
@@ -1771,32 +1754,32 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1808,12 +1791,12 @@
         <v>60</v>
       </c>
       <c r="E17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -1825,30 +1808,30 @@
         <v>53</v>
       </c>
       <c r="E18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" t="s">
         <v>65</v>
-      </c>
-      <c r="E19" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1862,7 +1845,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1876,57 +1859,57 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1948,7 +1931,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2">
         <v>2021</v>
@@ -2054,100 +2037,100 @@
         <v>39.226051152380791</v>
       </c>
       <c r="D2" s="9">
-        <f>'45Q Value'!C7*About!E31</f>
-        <v>64.04779095640987</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="E2" s="9">
-        <f>'45Q Value'!C8*About!E32</f>
-        <v>62.212860508337869</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="F2" s="9">
-        <f>'45Q Value'!C9*About!E33</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="G2" s="9">
-        <f>'45Q Value'!C10*About!E34</f>
-        <v>59.141100520738689</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="H2" s="9">
-        <f>$F$2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="I2" s="9">
-        <f t="shared" ref="I2:M2" si="0">H2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="J2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="K2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="L2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="M2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="N2" s="9">
         <f>$M2*(1-Calculations!N3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="O2" s="9">
         <f>$M2*(1-Calculations!O3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="P2" s="9">
         <f>$M2*(1-Calculations!P3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q2" s="9">
         <f>$M2*(1-Calculations!Q3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="R2" s="9">
         <f>$M2*(1-Calculations!R3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="S2" s="9">
         <f>$M2*(1-Calculations!S3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="T2" s="9">
         <f>$M2*(1-Calculations!T3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="U2" s="9">
         <f>$M2*(1-Calculations!U3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="V2" s="9">
         <f>$M2*(1-Calculations!V3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="W2" s="9">
         <f>$M2*(1-Calculations!W3)</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="X2" s="9">
         <f>$M2*(1-Calculations!X3)</f>
-        <v>48.526031196503546</v>
+        <v>48.491411999999997</v>
       </c>
       <c r="Y2" s="9">
         <f>$M2*(1-Calculations!Y3)</f>
-        <v>36.394523397377654</v>
+        <v>36.368558999999998</v>
       </c>
       <c r="Z2" s="9">
         <f>$M2*(1-Calculations!Z3)</f>
-        <v>24.263015598251766</v>
+        <v>24.245705999999991</v>
       </c>
       <c r="AA2" s="9">
         <f>$M2*(1-Calculations!AA3)</f>
-        <v>12.131507799125883</v>
+        <v>12.122852999999996</v>
       </c>
       <c r="AB2" s="9">
         <f>$M2*(1-Calculations!AB3)</f>
@@ -2184,7 +2167,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>87</v>
+        <v>6</v>
       </c>
       <c r="B1">
         <v>2021</v>
@@ -2279,7 +2262,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2374,7 +2357,7 @@
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2469,7 +2452,7 @@
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2564,7 +2547,7 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2659,7 +2642,7 @@
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2754,7 +2737,7 @@
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2849,7 +2832,7 @@
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2944,7 +2927,7 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -3039,7 +3022,7 @@
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -3134,7 +3117,7 @@
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -3229,7 +3212,7 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -3324,7 +3307,7 @@
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -3419,7 +3402,7 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -3514,7 +3497,7 @@
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -3609,7 +3592,7 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -3704,7 +3687,7 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -3799,7 +3782,7 @@
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -3894,7 +3877,7 @@
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B19" s="9">
         <f>'BCS-industry'!B2</f>
@@ -3905,53 +3888,56 @@
         <v>39.226051152380791</v>
       </c>
       <c r="D19" s="9">
-        <f>'BCS-industry'!D2</f>
-        <v>64.04779095640987</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="E19" s="9">
-        <f>'BCS-industry'!E2</f>
-        <v>62.212860508337869</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="F19" s="9">
-        <f>'BCS-industry'!F2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="G19" s="9">
-        <f>'BCS-industry'!G2</f>
-        <v>59.141100520738689</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="H19" s="9">
-        <f>'BCS-industry'!H2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="I19" s="9">
-        <f>'BCS-industry'!I2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="J19" s="9">
-        <f>'BCS-industry'!J2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="K19" s="9">
-        <f>'BCS-industry'!K2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="L19" s="9">
-        <f>'BCS-industry'!L2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="M19" s="9">
-        <f>'BCS-industry'!M2</f>
-        <v>60.65753899562943</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="O19">
-        <v>0</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="P19">
-        <v>0</v>
+        <f>About!$B$11*About!$A$9</f>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q19">
         <v>0</v>
@@ -4001,7 +3987,7 @@
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B20" s="11">
         <f>B19</f>
@@ -4013,55 +3999,55 @@
       </c>
       <c r="D20" s="11">
         <f t="shared" ref="D20:D22" si="1">D19</f>
-        <v>64.04779095640987</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="E20" s="11">
         <f t="shared" ref="E20:E22" si="2">E19</f>
-        <v>62.212860508337869</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="F20" s="11">
         <f t="shared" ref="F20:F22" si="3">F19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="G20" s="11">
         <f t="shared" ref="G20:G22" si="4">G19</f>
-        <v>59.141100520738689</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="H20" s="11">
         <f t="shared" ref="H20:H22" si="5">H19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="I20" s="11">
         <f t="shared" ref="I20:I22" si="6">I19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="J20" s="11">
         <f t="shared" ref="J20:J22" si="7">J19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="K20" s="11">
         <f t="shared" ref="K20:K22" si="8">K19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="L20" s="11">
         <f t="shared" ref="L20:L22" si="9">L19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="M20" s="11">
         <f t="shared" ref="M20:M22" si="10">M19</f>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="N20" s="11">
         <f t="shared" ref="N20:N22" si="11">N19</f>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="O20" s="11">
         <f t="shared" ref="O20:O22" si="12">O19</f>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="P20" s="11">
         <f t="shared" ref="P20:P22" si="13">P19</f>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q20" s="11">
         <f t="shared" ref="Q20:Q22" si="14">Q19</f>
@@ -4126,7 +4112,7 @@
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B21" s="11">
         <f t="shared" ref="B21:B22" si="29">B20</f>
@@ -4138,55 +4124,55 @@
       </c>
       <c r="D21" s="11">
         <f t="shared" si="1"/>
-        <v>64.04779095640987</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="E21" s="11">
         <f t="shared" si="2"/>
-        <v>62.212860508337869</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="F21" s="11">
         <f t="shared" si="3"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="G21" s="11">
         <f t="shared" si="4"/>
-        <v>59.141100520738689</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="H21" s="11">
         <f t="shared" si="5"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="I21" s="11">
         <f t="shared" si="6"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="J21" s="11">
         <f t="shared" si="7"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="K21" s="11">
         <f t="shared" si="8"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="L21" s="11">
         <f t="shared" si="9"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="M21" s="11">
         <f t="shared" si="10"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="N21" s="11">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="O21" s="11">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="P21" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q21" s="11">
         <f t="shared" si="14"/>
@@ -4251,7 +4237,7 @@
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B22" s="11">
         <f t="shared" si="29"/>
@@ -4263,55 +4249,55 @@
       </c>
       <c r="D22" s="11">
         <f t="shared" si="1"/>
-        <v>64.04779095640987</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="E22" s="11">
         <f t="shared" si="2"/>
-        <v>62.212860508337869</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="F22" s="11">
         <f t="shared" si="3"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="G22" s="11">
         <f t="shared" si="4"/>
-        <v>59.141100520738689</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="H22" s="11">
         <f t="shared" si="5"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="I22" s="11">
         <f t="shared" si="6"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="J22" s="11">
         <f t="shared" si="7"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="K22" s="11">
         <f t="shared" si="8"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="L22" s="11">
         <f t="shared" si="9"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="M22" s="11">
         <f t="shared" si="10"/>
-        <v>60.65753899562943</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="N22" s="11">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="O22" s="11">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="P22" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q22" s="11">
         <f t="shared" si="14"/>
@@ -4376,7 +4362,7 @@
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -4471,7 +4457,7 @@
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -4566,7 +4552,7 @@
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -4674,7 +4660,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1">
         <v>2021</v>
@@ -4769,7 +4755,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2">
         <v>12</v>

</xml_diff>